<commit_message>
chore(llm): adiciona script para conversão da planilha em CSV
</commit_message>
<xml_diff>
--- a/docs/llm/casos_de_teste.xlsx
+++ b/docs/llm/casos_de_teste.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\eduar\Documents\GitHub\PsicoCare\docs\llm\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ACE59ECA-0894-420B-8D23-89C376889DC4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B883B9C8-57D4-414B-8C90-363FDF83BD9C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -625,7 +625,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:N31"/>
+  <dimension ref="A1:N16"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="3.85546875" style="1" bestFit="1" customWidth="1"/>
@@ -1203,81 +1203,6 @@
         <v>79</v>
       </c>
     </row>
-    <row r="17" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A17" s="1">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="18" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A18" s="1">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="19" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A19" s="1">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="20" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A20" s="1">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="21" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A21" s="1">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="22" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A22" s="1">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="23" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A23" s="1">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="24" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A24" s="1">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="25" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A25" s="1">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="26" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A26" s="1">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="27" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A27" s="1">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="28" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A28" s="1">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="29" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A29" s="1">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="30" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A30" s="1">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="31" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A31" s="1">
-        <v>30</v>
-      </c>
-    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
test: add 31 LLM stress analysis validation cases
</commit_message>
<xml_diff>
--- a/docs/llm/casos_de_teste.xlsx
+++ b/docs/llm/casos_de_teste.xlsx
@@ -8,13 +8,16 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\eduar\Documents\GitHub\PsicoCare\docs\llm\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B883B9C8-57D4-414B-8C90-363FDF83BD9C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{067E592F-1F12-44D9-A8BB-D4AA3D38FB9D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Plan1" sheetId="1" r:id="rId1"/>
   </sheets>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Plan1!$A$1:$K$51</definedName>
+  </definedNames>
   <calcPr calcId="162913"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
@@ -25,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="161" uniqueCount="80">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="321" uniqueCount="139">
   <si>
     <t>ID</t>
   </si>
@@ -172,9 +175,6 @@
     <t>Recuperação</t>
   </si>
   <si>
-    <t>0.50–0.70</t>
-  </si>
-  <si>
     <t>Sentimento Real</t>
   </si>
   <si>
@@ -203,9 +203,6 @@
         "dificuldade"</t>
   </si>
   <si>
-    <t>0.45–0.65</t>
-  </si>
-  <si>
     <t>"Chorei bastante pela manhã, porém conversar com meus amigos me ajudou e agora estou mais tranquila."</t>
   </si>
   <si>
@@ -231,9 +228,6 @@
     <t>"Passei o dia inteiro chorando. Não consegui trabalhar e me sinto completamente sobrecarregada."</t>
   </si>
   <si>
-    <t>0.90–1.00</t>
-  </si>
-  <si>
     <t xml:space="preserve">        "estresse",
         "sobrecarga",
         "tristeza"</t>
@@ -258,9 +252,6 @@
     <t>Verificar a identificação de relatos com sinais claros de estresse intenso.</t>
   </si>
   <si>
-    <t xml:space="preserve">Alto </t>
-  </si>
-  <si>
     <t>A LLM atribuiu um nível moderado de estresse ao relato, reconhecendo a ansiedade inicial, mas também considerando o fator de recuperação descrito após a conversa com a terapeuta. O resultado foi compatível com o comportamento esperado.</t>
   </si>
   <si>
@@ -277,9 +268,6 @@
   </si>
   <si>
     <t>A LLM identificou corretamente um relato de alto estresse, marcado por ansiedade intensa e sensação de incapacidade para lidar com a pressão. O stress_score máximo foi compatível com a gravidade descrita.</t>
-  </si>
-  <si>
-    <t>Casos exploratórios</t>
   </si>
   <si>
     <t>Avaliar o comportamento da LLM em situações emocionalmente negativas que não representam necessariamente um quadro de estresse.</t>
@@ -294,6 +282,228 @@
   </si>
   <si>
     <t>O modelo atribuiu stress_score = 1.0 ao relato de luto. Embora o sentimento negativo seja coerente, o resultado sugere que a LLM pode associar eventos de grande impacto emocional diretamente a níveis máximos de estresse. Esse comportamento deverá ser discutido como uma limitação ou característica do modelo.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Muito Alto </t>
+  </si>
+  <si>
+    <t>Leve</t>
+  </si>
+  <si>
+    <t>Verificar se a LLM identifica pequenas preocupações cotidianas sem superestimar sua intensidade.</t>
+  </si>
+  <si>
+    <t>0.20–0.40</t>
+  </si>
+  <si>
+    <t>Fiquei um pouco preocupada porque tenho algumas tarefas para terminar amanhã, mas consegui fazer tudo normalmente hoje e estou tranquila</t>
+  </si>
+  <si>
+    <t>Positivo ou neutro</t>
+  </si>
+  <si>
+    <t>Neutro</t>
+  </si>
+  <si>
+    <t xml:space="preserve">        "tranquila",
+        "preocupada",
+        "trabalho"</t>
+  </si>
+  <si>
+    <t>Me atrasei para um compromisso hoje e fiquei um pouco nervosa, mas no final deu tudo certo e consegui seguir meu dia normalmente.</t>
+  </si>
+  <si>
+    <t>0.20</t>
+  </si>
+  <si>
+    <t xml:space="preserve">        "nervosa",
+        "sucedido",
+        "normalmente"</t>
+  </si>
+  <si>
+    <t>Tive um pequeno problema no trabalho que me deixou irritada por um tempo, mas consegui resolver e depois continuei minhas atividades normalmente</t>
+  </si>
+  <si>
+    <t>Hoje fiquei um pouco cansada porque tive mais coisas para fazer do que o normal, mas consegui organizar tudo e não tive grandes dificuldades.</t>
+  </si>
+  <si>
+    <t>Tenho uma prova chegando e estou um pouco preocupada porque ainda preciso estudar algumas coisas, mas estou conseguindo me organizar e acho que vai dar tudo certo.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">        "cansada",
+        "organizar",
+        "dificuldades"</t>
+  </si>
+  <si>
+    <t xml:space="preserve">        "irritada",
+        "problema",
+        "trabalho"</t>
+  </si>
+  <si>
+    <t xml:space="preserve">        "preocupação",
+        "estresse",
+        "ansiedade"</t>
+  </si>
+  <si>
+    <t>Não</t>
+  </si>
+  <si>
+    <t>A LLM identificou adequadamente um nível leve de estresse, atribuindo stress_score de 0,30 diante de uma preocupação pontual sem comprometimento das atividades diárias. O sentimento positivo é coerente com a tranquilidade relatada ao final do texto, e as palavras-chave representam tanto a preocupação quanto o estado de tranquilidade descrito.</t>
+  </si>
+  <si>
+    <t>O modelo classificou adequadamente a situação como estresse leve, com stress_score de 0,20. Apesar do nervosismo causado pelo atraso, o relato descreve resolução do imprevisto e continuidade normal das atividades. O sentimento positivo e as palavras-chave retornadas refletem a recuperação e o desfecho favorável da situação.</t>
+  </si>
+  <si>
+    <t>A LLM atribuiu stress_score de 0,30, compatível com a faixa de estresse leve. O sentimento negativo é coerente com a irritação explicitamente relatada, enquanto a resolução do problema e a manutenção das atividades indicam ausência de impacto funcional significativo. As palavras-chave representam adequadamente o principal fator de tensão descrito.</t>
+  </si>
+  <si>
+    <t>O modelo identificou corretamente um nível leve de estresse, com stress_score de 0,20. O relato apresenta cansaço e aumento pontual de demanda, porém sem dificuldades significativas ou prejuízo no funcionamento diário. A classificação neutra do sentimento e as palavras-chave retornadas foram consideradas coerentes com o conteúdo apresentado.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">        "preocupação",
+        "estresse",
+        "dificuldade"</t>
+  </si>
+  <si>
+    <t>Passei boa parte do dia preocupada com alguns problemas pessoais e tive dificuldade para me concentrar. Mesmo assim, consegui terminar minhas principais tarefas e seguir com o meu dia.</t>
+  </si>
+  <si>
+    <t>A LLM identificou adequadamente um nível moderado de estresse, atribuindo stress_score de 0,50 diante da preocupação antecipatória relacionada à prova e às demandas de estudo. Apesar da presença de fatores de controle, como organização e expectativa positiva de resolução, o modelo reconheceu a preocupação como elemento relevante de estresse. O sentimento negativo e as palavras-chave retornadas foram coerentes com o conteúdo do relato.</t>
+  </si>
+  <si>
+    <t>A LLM identificou corretamente um nível moderado de estresse, com stress_score de 0,50. O relato apresenta preocupação persistente e dificuldade de concentração, indicando impacto perceptível no cotidiano, porém sem comprometimento significativo do funcionamento, uma vez que as principais tarefas foram concluídas. O sentimento negativo e as palavras-chave retornadas foram coerentes com os fatores de estresse descritos.</t>
+  </si>
+  <si>
+    <t>0.3</t>
+  </si>
+  <si>
+    <t>Hoje fiquei um pouco incomodada porque precisei refazer uma tarefa que já tinha terminado. Foi chato perder esse tempo, mas resolvi sem grandes dificuldades e segui meu dia normalmente.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">        "incomodada",
+        "perder",
+        "chato"</t>
+  </si>
+  <si>
+    <t>A LLM identificou adequadamente um nível leve de estresse, atribuindo stress_score de 0,30 diante de um incômodo pontual relacionado à necessidade de refazer uma tarefa. O sentimento negativo e as palavras-chave retornadas foram coerentes com a frustração descrita, enquanto a resolução do problema sem grandes dificuldades e a continuidade normal das atividades indicam ausência de impacto funcional significativo. O resultado foi compatível com a faixa esperada de estresse leve.</t>
+  </si>
+  <si>
+    <t>Alto</t>
+  </si>
+  <si>
+    <t>0.60–0.80</t>
+  </si>
+  <si>
+    <t>Verificar se a LLM identifica estresse elevado quando a sobrecarga começa a comprometer o desempenho diário.</t>
+  </si>
+  <si>
+    <t>Estou com muitas demandas acumuladas no trabalho e está ficando difícil acompanhar tudo. Hoje não consegui terminar algumas tarefas e passei boa parte do dia preocupada com o que ficou pendente.</t>
+  </si>
+  <si>
+    <t>"demanda",
+        "preocupação",
+        "estresse"</t>
+  </si>
+  <si>
+    <t>Estou muito preocupada com alguns problemas pessoais e isso está afetando meu dia. Tive bastante dificuldade para me concentrar no trabalho e produzi bem menos do que normalmente consigo.</t>
+  </si>
+  <si>
+    <t>Tenho me sentido muito sobrecarregada nos últimos dias. Estou constantemente cansada e hoje precisei adiar algumas atividades porque estava difícil manter o ritmo.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">        "sobrecarregada",
+        "cansada",
+        "estresse"</t>
+  </si>
+  <si>
+    <t>Estou muito nervosa com as provas e trabalhos acumulados. Tentei estudar hoje, mas minha preocupação atrapalhou bastante e consegui avançar muito menos do que precisava.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">        "nervosa",
+        "preocupação",
+        "estresse"</t>
+  </si>
+  <si>
+    <t>O trabalho está me deixando muito tensa. Mesmo depois de chegar em casa, continuo pensando nos problemas e estou tendo bastante dificuldade para relaxar e aproveitar meu tempo de descanso.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">        "tensa",
+        "estresse",
+        "dificuldade"</t>
+  </si>
+  <si>
+    <t>A LLM identificou adequadamente um nível alto de estresse, atribuindo stress_score de 0,80 diante da presença de demandas acumuladas, preocupação persistente e prejuízo no desempenho diário, evidenciado pela dificuldade em concluir algumas tarefas. O sentimento negativo e as palavras-chave retornadas foram coerentes com os fatores de sobrecarga presentes no relato.</t>
+  </si>
+  <si>
+    <t>O modelo identificou corretamente um nível alto de estresse, com stress_score de 0,80. O relato apresenta preocupação significativa acompanhada de dificuldade de concentração e redução da produtividade, indicando impacto relevante no funcionamento diário. O sentimento negativo e as palavras-chave foram compatíveis com o conteúdo apresentado.</t>
+  </si>
+  <si>
+    <t>A LLM atribuiu stress_score de 0,50, abaixo da faixa esperada para estresse alto e correspondente à categoria moderada. Embora o modelo tenha identificado corretamente o sentimento negativo e elementos relevantes de sobrecarga e cansaço, o score sugere que o impacto funcional descrito pelo adiamento de atividades não foi suficiente para que o modelo classificasse o relato na intensidade esperada. O resultado indica possível subestimação do estresse em situações de sobrecarga e cansaço persistentes sem manifestações emocionais mais intensas.</t>
+  </si>
+  <si>
+    <t>A LLM identificou adequadamente um nível alto de estresse, atribuindo stress_score de 0,80 diante da pressão acadêmica, do nervosismo e da interferência da preocupação no desempenho dos estudos. O sentimento negativo e as palavras-chave retornadas foram coerentes com a intensidade e os fatores de estresse descritos.</t>
+  </si>
+  <si>
+    <t>O modelo classificou adequadamente o relato como estresse alto, com stress_score de 0,80. A persistência da preocupação após o período de trabalho e a dificuldade significativa para relaxar indicam interferência do estresse no período de descanso. O sentimento negativo e as palavras-chave retornadas foram coerentes com o conteúdo do relato.</t>
+  </si>
+  <si>
+    <t>Estou me sentindo completamente sobrecarregada. Hoje fiquei tão nervosa que comecei a tremer e senti meu coração muito acelerado. Precisei parar o que estava fazendo porque não conseguia continuar.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">        "sobrecarregada",
+        "nervosa",
+        "ansiedade"</t>
+  </si>
+  <si>
+    <t>Sinto que cheguei ao meu limite com tudo que está acontecendo. Hoje não consegui me concentrar em praticamente nada, abandonei várias tarefas e passei grande parte do dia angustiada e sem conseguir me acalmar.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">        "estresse",
+        "angustiada",
+        "sobrecarga"</t>
+  </si>
+  <si>
+    <t>A LLM identificou adequadamente um nível muito alto de estresse, atribuindo stress_score de 1,00 diante da combinação de sobrecarga intensa, nervosismo, sintomas físicos e comprometimento funcional, evidenciado pela necessidade de interromper a atividade que estava sendo realizada. O sentimento negativo e as palavras-chave retornadas foram coerentes com a intensidade do estresse descrito.</t>
+  </si>
+  <si>
+    <t>O modelo identificou corretamente um nível muito alto de estresse, com stress_score de 1,00. O relato apresenta sensação de limite, angústia persistente, dificuldade significativa de concentração, abandono de tarefas e incapacidade de se acalmar, indicando comprometimento importante do funcionamento diário. O sentimento negativo e as palavras-chave retornadas foram compatíveis com a gravidade do relato.</t>
+  </si>
+  <si>
+    <t>Exploratórios</t>
+  </si>
+  <si>
+    <t>Avaliar se a LLM diferencia emoção positiva de alta intensidade de um quadro de estresse.</t>
+  </si>
+  <si>
+    <t>Avaliar o comportamento da LLM diante de uma emoção negativa intensa causada por um evento pontual, sem evidências explícitas de sobrecarga ou estresse.</t>
+  </si>
+  <si>
+    <t>Sem faixa pré-definida</t>
+  </si>
+  <si>
+    <t>"Hoje recebi a notícia de que fui aprovada em uma oportunidade que eu queria muito. Meu coração disparou, comecei a chorar e fiquei tão emocionada que mal conseguia ficar parada."</t>
+  </si>
+  <si>
+    <t>“Assisti a um filme muito triste hoje e chorei bastante com o final. Fiquei emocionada por um tempo, mas foi só por causa da história.”</t>
+  </si>
+  <si>
+    <t xml:space="preserve">        "triste",
+        "emocionada",
+        "chorei"</t>
+  </si>
+  <si>
+    <t xml:space="preserve">        "emocionada",
+        "alegria",
+        "satisfação"</t>
+  </si>
+  <si>
+    <t>A LLM atribuiu stress_score de 0,00 ao relato, apesar da presença de sinais de elevada ativação emocional, como aceleração cardíaca, choro e agitação. O resultado indica que o modelo considerou adequadamente o contexto positivo da narrativa, diferenciando excitação emocional de estresse. O sentimento positivo e as palavras-chave retornadas foram coerentes com a experiência de alegria e satisfação descrita.</t>
+  </si>
+  <si>
+    <t>A LLM atribuiu stress_score de 0,50 ao relato de tristeza provocada por um filme, apesar da ausência de um estressor pessoal ou de prejuízo funcional. Embora o sentimento negativo e as palavras-chave sejam coerentes com a emoção descrita, o score moderado sugere que o modelo pode atribuir estresse a manifestações de emoção negativa intensa, como tristeza e choro, mesmo quando o contexto não indica necessariamente uma situação de estresse. O resultado reforça uma possível limitação do modelo na diferenciação entre intensidade emocional negativa e estresse percebido.</t>
+  </si>
+  <si>
+    <t>Sim/Não</t>
   </si>
 </sst>
 </file>
@@ -337,12 +547,15 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -625,24 +838,24 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:N16"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:N32"/>
+  <sheetFormatPr defaultColWidth="24.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="3.85546875" style="1" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="18.140625" style="1" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="29.28515625" style="1" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="53.28515625" style="1" customWidth="1"/>
-    <col min="5" max="5" width="14.7109375" style="1" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="12.140625" style="1" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="12.140625" style="1" customWidth="1"/>
-    <col min="8" max="8" width="12.140625" style="1" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="20.42578125" style="1" customWidth="1"/>
-    <col min="10" max="10" width="8.140625" style="1" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="64.42578125" style="1" customWidth="1"/>
-    <col min="12" max="16384" width="9.140625" style="1"/>
+    <col min="1" max="1" width="12.140625" style="1" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="19.42578125" style="1" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="35.42578125" style="1" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="52.140625" style="1" customWidth="1"/>
+    <col min="5" max="5" width="24.5703125" style="1" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="19.42578125" style="1" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="30" style="1" customWidth="1"/>
+    <col min="8" max="8" width="25.140625" style="1" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="23.7109375" style="1" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="18" style="1" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="83.5703125" style="1" bestFit="1" customWidth="1"/>
+    <col min="12" max="16384" width="24.85546875" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:14" ht="30" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -656,16 +869,16 @@
         <v>3</v>
       </c>
       <c r="E1" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="F1" s="1" t="s">
         <v>46</v>
       </c>
-      <c r="F1" s="1" t="s">
-        <v>47</v>
-      </c>
       <c r="G1" s="1" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="I1" s="1" t="s">
         <v>4</v>
@@ -685,7 +898,7 @@
         <v>29</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>64</v>
+        <v>61</v>
       </c>
       <c r="D2" s="1" t="s">
         <v>6</v>
@@ -720,7 +933,7 @@
         <v>29</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>64</v>
+        <v>61</v>
       </c>
       <c r="D3" s="1" t="s">
         <v>12</v>
@@ -755,7 +968,7 @@
         <v>29</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>64</v>
+        <v>61</v>
       </c>
       <c r="D4" s="1" t="s">
         <v>14</v>
@@ -790,7 +1003,7 @@
         <v>29</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>64</v>
+        <v>61</v>
       </c>
       <c r="D5" s="1" t="s">
         <v>16</v>
@@ -825,7 +1038,7 @@
         <v>29</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>64</v>
+        <v>61</v>
       </c>
       <c r="D6" s="1" t="s">
         <v>18</v>
@@ -852,7 +1065,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="7" spans="1:14" ht="60" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:14" ht="45" x14ac:dyDescent="0.25">
       <c r="A7" s="1">
         <v>6</v>
       </c>
@@ -860,13 +1073,13 @@
         <v>30</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>65</v>
+        <v>62</v>
       </c>
       <c r="D7" s="1" t="s">
         <v>20</v>
       </c>
       <c r="E7" s="1" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="F7" s="1" t="s">
         <v>39</v>
@@ -887,7 +1100,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="8" spans="1:14" ht="75" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:14" ht="90" x14ac:dyDescent="0.25">
       <c r="A8" s="1">
         <v>7</v>
       </c>
@@ -895,16 +1108,16 @@
         <v>30</v>
       </c>
       <c r="C8" s="1" t="s">
-        <v>65</v>
+        <v>62</v>
       </c>
       <c r="D8" s="1" t="s">
-        <v>24</v>
+        <v>88</v>
       </c>
       <c r="E8" s="1" t="s">
         <v>25</v>
       </c>
       <c r="F8" s="1" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="G8" s="1" t="s">
         <v>22</v>
@@ -913,16 +1126,16 @@
         <v>22</v>
       </c>
       <c r="I8" s="1" t="s">
-        <v>26</v>
+        <v>91</v>
       </c>
       <c r="J8" s="1" t="s">
         <v>11</v>
       </c>
       <c r="K8" s="1" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="9" spans="1:14" ht="60" x14ac:dyDescent="0.25">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="9" spans="1:14" ht="90" x14ac:dyDescent="0.25">
       <c r="A9" s="1">
         <v>8</v>
       </c>
@@ -930,13 +1143,13 @@
         <v>30</v>
       </c>
       <c r="C9" s="1" t="s">
-        <v>65</v>
+        <v>62</v>
       </c>
       <c r="D9" s="1" t="s">
-        <v>27</v>
+        <v>98</v>
       </c>
       <c r="E9" s="1" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="F9" s="1" t="s">
         <v>39</v>
@@ -948,33 +1161,33 @@
         <v>22</v>
       </c>
       <c r="I9" s="1" t="s">
-        <v>28</v>
+        <v>97</v>
       </c>
       <c r="J9" s="1" t="s">
         <v>11</v>
       </c>
       <c r="K9" s="1" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="10" spans="1:14" ht="75" x14ac:dyDescent="0.25">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="10" spans="1:14" ht="60" x14ac:dyDescent="0.25">
       <c r="A10" s="1">
         <v>9</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>42</v>
+        <v>30</v>
       </c>
       <c r="C10" s="1" t="s">
-        <v>66</v>
+        <v>62</v>
       </c>
       <c r="D10" s="1" t="s">
-        <v>49</v>
+        <v>24</v>
       </c>
       <c r="E10" s="1" t="s">
-        <v>43</v>
+        <v>25</v>
       </c>
       <c r="F10" s="1" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="G10" s="1" t="s">
         <v>22</v>
@@ -983,30 +1196,30 @@
         <v>22</v>
       </c>
       <c r="I10" s="1" t="s">
-        <v>48</v>
+        <v>26</v>
       </c>
       <c r="J10" s="1" t="s">
-        <v>11</v>
+        <v>92</v>
       </c>
       <c r="K10" s="1" t="s">
-        <v>69</v>
-      </c>
-    </row>
-    <row r="11" spans="1:14" ht="75" x14ac:dyDescent="0.25">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="11" spans="1:14" ht="45" x14ac:dyDescent="0.25">
       <c r="A11" s="1">
         <v>10</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>42</v>
+        <v>30</v>
       </c>
       <c r="C11" s="1" t="s">
-        <v>66</v>
+        <v>62</v>
       </c>
       <c r="D11" s="1" t="s">
-        <v>50</v>
+        <v>27</v>
       </c>
       <c r="E11" s="1" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="F11" s="1" t="s">
         <v>39</v>
@@ -1018,16 +1231,16 @@
         <v>22</v>
       </c>
       <c r="I11" s="1" t="s">
-        <v>51</v>
+        <v>28</v>
       </c>
       <c r="J11" s="1" t="s">
         <v>11</v>
       </c>
       <c r="K11" s="1" t="s">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="12" spans="1:14" ht="75" x14ac:dyDescent="0.25">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="12" spans="1:14" ht="60" x14ac:dyDescent="0.25">
       <c r="A12" s="1">
         <v>11</v>
       </c>
@@ -1035,13 +1248,13 @@
         <v>42</v>
       </c>
       <c r="C12" s="1" t="s">
-        <v>66</v>
+        <v>63</v>
       </c>
       <c r="D12" s="1" t="s">
-        <v>53</v>
+        <v>48</v>
       </c>
       <c r="E12" s="1" t="s">
-        <v>52</v>
+        <v>21</v>
       </c>
       <c r="F12" s="1" t="s">
         <v>39</v>
@@ -1053,13 +1266,13 @@
         <v>22</v>
       </c>
       <c r="I12" s="1" t="s">
-        <v>54</v>
+        <v>47</v>
       </c>
       <c r="J12" s="1" t="s">
         <v>11</v>
       </c>
       <c r="K12" s="1" t="s">
-        <v>71</v>
+        <v>65</v>
       </c>
     </row>
     <row r="13" spans="1:14" ht="60" x14ac:dyDescent="0.25">
@@ -1067,19 +1280,19 @@
         <v>12</v>
       </c>
       <c r="B13" s="1" t="s">
-        <v>68</v>
+        <v>42</v>
       </c>
       <c r="C13" s="1" t="s">
-        <v>67</v>
+        <v>63</v>
       </c>
       <c r="D13" s="1" t="s">
-        <v>56</v>
+        <v>49</v>
       </c>
       <c r="E13" s="1" t="s">
-        <v>55</v>
+        <v>21</v>
       </c>
       <c r="F13" s="1" t="s">
-        <v>57</v>
+        <v>39</v>
       </c>
       <c r="G13" s="1" t="s">
         <v>22</v>
@@ -1088,13 +1301,13 @@
         <v>22</v>
       </c>
       <c r="I13" s="1" t="s">
-        <v>58</v>
+        <v>50</v>
       </c>
       <c r="J13" s="1" t="s">
         <v>11</v>
       </c>
       <c r="K13" s="1" t="s">
-        <v>72</v>
+        <v>66</v>
       </c>
     </row>
     <row r="14" spans="1:14" ht="60" x14ac:dyDescent="0.25">
@@ -1102,73 +1315,72 @@
         <v>13</v>
       </c>
       <c r="B14" s="1" t="s">
-        <v>68</v>
+        <v>42</v>
       </c>
       <c r="C14" s="1" t="s">
+        <v>63</v>
+      </c>
+      <c r="D14" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="E14" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="F14" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="G14" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="H14" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="I14" s="1" t="s">
+        <v>52</v>
+      </c>
+      <c r="J14" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="K14" s="1" t="s">
         <v>67</v>
       </c>
-      <c r="D14" s="1" t="s">
-        <v>59</v>
-      </c>
-      <c r="E14" s="1" t="s">
-        <v>60</v>
-      </c>
-      <c r="F14" s="1" t="s">
-        <v>63</v>
-      </c>
-      <c r="G14" s="1" t="s">
-        <v>22</v>
-      </c>
-      <c r="H14" s="1" t="s">
-        <v>22</v>
-      </c>
-      <c r="I14" s="1" t="s">
-        <v>61</v>
-      </c>
-      <c r="J14" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="K14" s="1" t="s">
-        <v>73</v>
-      </c>
-      <c r="N14" s="2"/>
-    </row>
-    <row r="15" spans="1:14" ht="60" x14ac:dyDescent="0.25">
+    </row>
+    <row r="15" spans="1:14" ht="45" x14ac:dyDescent="0.25">
       <c r="A15" s="1">
         <v>14</v>
       </c>
       <c r="B15" s="1" t="s">
+        <v>75</v>
+      </c>
+      <c r="C15" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="D15" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="E15" s="1" t="s">
+        <v>53</v>
+      </c>
+      <c r="F15" s="1" t="s">
+        <v>55</v>
+      </c>
+      <c r="G15" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="H15" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="I15" s="1" t="s">
+        <v>56</v>
+      </c>
+      <c r="J15" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="K15" s="1" t="s">
         <v>68</v>
       </c>
-      <c r="C15" s="1" t="s">
-        <v>67</v>
-      </c>
-      <c r="D15" s="1" t="s">
-        <v>62</v>
-      </c>
-      <c r="E15" s="1" t="s">
-        <v>55</v>
-      </c>
-      <c r="F15" s="1" t="s">
-        <v>63</v>
-      </c>
-      <c r="G15" s="1" t="s">
-        <v>22</v>
-      </c>
-      <c r="H15" s="1" t="s">
-        <v>22</v>
-      </c>
-      <c r="I15" s="1" t="s">
-        <v>61</v>
-      </c>
-      <c r="J15" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="K15" s="1" t="s">
-        <v>74</v>
-      </c>
-    </row>
-    <row r="16" spans="1:14" ht="90" x14ac:dyDescent="0.25">
+    </row>
+    <row r="16" spans="1:14" ht="45" x14ac:dyDescent="0.25">
       <c r="A16" s="1">
         <v>15</v>
       </c>
@@ -1176,34 +1388,599 @@
         <v>75</v>
       </c>
       <c r="C16" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="D16" s="1" t="s">
+        <v>57</v>
+      </c>
+      <c r="E16" s="1" t="s">
+        <v>53</v>
+      </c>
+      <c r="F16" s="1" t="s">
+        <v>60</v>
+      </c>
+      <c r="G16" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="H16" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="I16" s="1" t="s">
+        <v>58</v>
+      </c>
+      <c r="J16" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="K16" s="1" t="s">
+        <v>69</v>
+      </c>
+      <c r="N16" s="2"/>
+    </row>
+    <row r="17" spans="1:14" ht="75" x14ac:dyDescent="0.25">
+      <c r="A17" s="1">
+        <v>16</v>
+      </c>
+      <c r="B17" s="1" t="s">
+        <v>75</v>
+      </c>
+      <c r="C17" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="D17" s="1" t="s">
+        <v>122</v>
+      </c>
+      <c r="E17" s="1" t="s">
+        <v>53</v>
+      </c>
+      <c r="F17" s="1" t="s">
+        <v>60</v>
+      </c>
+      <c r="G17" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="H17" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="I17" s="1" t="s">
+        <v>123</v>
+      </c>
+      <c r="J17" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="K17" s="1" t="s">
+        <v>126</v>
+      </c>
+      <c r="N17" s="2"/>
+    </row>
+    <row r="18" spans="1:14" ht="75" x14ac:dyDescent="0.25">
+      <c r="A18" s="1">
+        <v>17</v>
+      </c>
+      <c r="B18" s="1" t="s">
+        <v>75</v>
+      </c>
+      <c r="C18" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="D18" s="1" t="s">
+        <v>124</v>
+      </c>
+      <c r="E18" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="F18" s="1" t="s">
+        <v>60</v>
+      </c>
+      <c r="G18" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="H18" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="I18" s="1" t="s">
+        <v>125</v>
+      </c>
+      <c r="J18" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="K18" s="1" t="s">
+        <v>127</v>
+      </c>
+      <c r="N18" s="2"/>
+    </row>
+    <row r="19" spans="1:14" ht="45" x14ac:dyDescent="0.25">
+      <c r="A19" s="1">
+        <v>18</v>
+      </c>
+      <c r="B19" s="1" t="s">
+        <v>75</v>
+      </c>
+      <c r="C19" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="D19" s="1" t="s">
+        <v>59</v>
+      </c>
+      <c r="E19" s="1" t="s">
+        <v>53</v>
+      </c>
+      <c r="F19" s="1" t="s">
+        <v>60</v>
+      </c>
+      <c r="G19" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="H19" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="I19" s="1" t="s">
+        <v>58</v>
+      </c>
+      <c r="J19" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="K19" s="1" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="20" spans="1:14" ht="75" x14ac:dyDescent="0.25">
+      <c r="A20" s="1">
+        <v>19</v>
+      </c>
+      <c r="B20" s="1" t="s">
+        <v>128</v>
+      </c>
+      <c r="C20" s="1" t="s">
+        <v>129</v>
+      </c>
+      <c r="D20" s="1" t="s">
+        <v>132</v>
+      </c>
+      <c r="E20" s="1" t="s">
+        <v>131</v>
+      </c>
+      <c r="F20" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="G20" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="H20" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="I20" s="1" t="s">
+        <v>135</v>
+      </c>
+      <c r="J20" s="1" t="s">
+        <v>138</v>
+      </c>
+      <c r="K20" s="1" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="21" spans="1:14" ht="105" x14ac:dyDescent="0.25">
+      <c r="A21" s="1">
+        <v>20</v>
+      </c>
+      <c r="B21" s="1" t="s">
+        <v>128</v>
+      </c>
+      <c r="C21" s="1" t="s">
+        <v>130</v>
+      </c>
+      <c r="D21" s="1" t="s">
+        <v>133</v>
+      </c>
+      <c r="E21" s="1" t="s">
+        <v>131</v>
+      </c>
+      <c r="F21" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="G21" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="H21" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="I21" s="1" t="s">
+        <v>134</v>
+      </c>
+      <c r="J21" s="1" t="s">
+        <v>138</v>
+      </c>
+      <c r="K21" s="1" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="22" spans="1:14" ht="75" x14ac:dyDescent="0.25">
+      <c r="A22" s="1">
+        <v>21</v>
+      </c>
+      <c r="B22" s="1" t="s">
+        <v>128</v>
+      </c>
+      <c r="C22" s="1" t="s">
+        <v>71</v>
+      </c>
+      <c r="D22" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="E22" s="1" t="s">
+        <v>131</v>
+      </c>
+      <c r="F22" s="1" t="s">
+        <v>60</v>
+      </c>
+      <c r="G22" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="H22" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="I22" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="J22" s="1" t="s">
+        <v>138</v>
+      </c>
+      <c r="K22" s="1" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="23" spans="1:14" ht="75" x14ac:dyDescent="0.25">
+      <c r="A23" s="1">
+        <v>22</v>
+      </c>
+      <c r="B23" s="1" t="s">
         <v>76</v>
       </c>
-      <c r="D16" s="1" t="s">
+      <c r="C23" s="1" t="s">
         <v>77</v>
       </c>
-      <c r="E16" s="1" t="s">
+      <c r="D23" s="1" t="s">
+        <v>79</v>
+      </c>
+      <c r="E23" s="1" t="s">
+        <v>78</v>
+      </c>
+      <c r="F23" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="G23" s="1" t="s">
+        <v>80</v>
+      </c>
+      <c r="H23" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="I23" s="1" t="s">
+        <v>82</v>
+      </c>
+      <c r="J23" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="K23" s="1" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="24" spans="1:14" ht="60" x14ac:dyDescent="0.25">
+      <c r="A24" s="1">
+        <v>23</v>
+      </c>
+      <c r="B24" s="1" t="s">
+        <v>76</v>
+      </c>
+      <c r="C24" s="1" t="s">
+        <v>77</v>
+      </c>
+      <c r="D24" s="1" t="s">
+        <v>83</v>
+      </c>
+      <c r="E24" s="1" t="s">
+        <v>78</v>
+      </c>
+      <c r="F24" s="1" t="s">
+        <v>84</v>
+      </c>
+      <c r="G24" s="1" t="s">
+        <v>80</v>
+      </c>
+      <c r="H24" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="I24" s="1" t="s">
+        <v>85</v>
+      </c>
+      <c r="J24" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="K24" s="1" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="25" spans="1:14" ht="75" x14ac:dyDescent="0.25">
+      <c r="A25" s="1">
+        <v>24</v>
+      </c>
+      <c r="B25" s="1" t="s">
+        <v>76</v>
+      </c>
+      <c r="C25" s="1" t="s">
+        <v>77</v>
+      </c>
+      <c r="D25" s="1" t="s">
+        <v>86</v>
+      </c>
+      <c r="E25" s="1" t="s">
+        <v>78</v>
+      </c>
+      <c r="F25" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="G25" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="H25" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="I25" s="1" t="s">
+        <v>90</v>
+      </c>
+      <c r="J25" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="K25" s="1" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="26" spans="1:14" ht="60" x14ac:dyDescent="0.25">
+      <c r="A26" s="1">
+        <v>25</v>
+      </c>
+      <c r="B26" s="1" t="s">
+        <v>76</v>
+      </c>
+      <c r="C26" s="1" t="s">
+        <v>77</v>
+      </c>
+      <c r="D26" s="1" t="s">
+        <v>87</v>
+      </c>
+      <c r="E26" s="1" t="s">
+        <v>78</v>
+      </c>
+      <c r="F26" s="1" t="s">
+        <v>84</v>
+      </c>
+      <c r="G26" s="1" t="s">
+        <v>81</v>
+      </c>
+      <c r="H26" s="1" t="s">
+        <v>81</v>
+      </c>
+      <c r="I26" s="1" t="s">
+        <v>89</v>
+      </c>
+      <c r="J26" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="K26" s="1" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="27" spans="1:14" ht="90" x14ac:dyDescent="0.25">
+      <c r="A27" s="1">
+        <v>26</v>
+      </c>
+      <c r="B27" s="1" t="s">
+        <v>76</v>
+      </c>
+      <c r="C27" s="1" t="s">
+        <v>77</v>
+      </c>
+      <c r="D27" s="1" t="s">
+        <v>102</v>
+      </c>
+      <c r="E27" s="1" t="s">
+        <v>78</v>
+      </c>
+      <c r="F27" s="1" t="s">
+        <v>101</v>
+      </c>
+      <c r="G27" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="H27" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="I27" s="1" t="s">
+        <v>103</v>
+      </c>
+      <c r="J27" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="K27" s="1" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="28" spans="1:14" ht="75" x14ac:dyDescent="0.25">
+      <c r="A28" s="1">
+        <v>27</v>
+      </c>
+      <c r="B28" s="1" t="s">
+        <v>105</v>
+      </c>
+      <c r="C28" s="1" t="s">
+        <v>107</v>
+      </c>
+      <c r="D28" s="1" t="s">
+        <v>108</v>
+      </c>
+      <c r="E28" s="1" t="s">
+        <v>106</v>
+      </c>
+      <c r="F28" s="1" t="s">
         <v>55</v>
       </c>
-      <c r="F16" s="1" t="s">
-        <v>63</v>
-      </c>
-      <c r="G16" s="1" t="s">
-        <v>22</v>
-      </c>
-      <c r="H16" s="1" t="s">
-        <v>22</v>
-      </c>
-      <c r="I16" s="1" t="s">
-        <v>78</v>
-      </c>
-      <c r="J16" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="K16" s="1" t="s">
-        <v>79</v>
+      <c r="G28" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="H28" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="I28" s="1" t="s">
+        <v>109</v>
+      </c>
+      <c r="J28" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="K28" s="1" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="29" spans="1:14" ht="60" x14ac:dyDescent="0.25">
+      <c r="A29" s="1">
+        <v>28</v>
+      </c>
+      <c r="B29" s="1" t="s">
+        <v>105</v>
+      </c>
+      <c r="C29" s="1" t="s">
+        <v>107</v>
+      </c>
+      <c r="D29" s="1" t="s">
+        <v>110</v>
+      </c>
+      <c r="E29" s="1" t="s">
+        <v>106</v>
+      </c>
+      <c r="F29" s="1" t="s">
+        <v>55</v>
+      </c>
+      <c r="G29" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="H29" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="I29" s="1" t="s">
+        <v>97</v>
+      </c>
+      <c r="J29" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="K29" s="1" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="30" spans="1:14" ht="105" x14ac:dyDescent="0.25">
+      <c r="A30" s="1">
+        <v>29</v>
+      </c>
+      <c r="B30" s="1" t="s">
+        <v>105</v>
+      </c>
+      <c r="C30" s="1" t="s">
+        <v>107</v>
+      </c>
+      <c r="D30" s="1" t="s">
+        <v>111</v>
+      </c>
+      <c r="E30" s="1" t="s">
+        <v>106</v>
+      </c>
+      <c r="F30" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="G30" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="H30" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="I30" s="1" t="s">
+        <v>112</v>
+      </c>
+      <c r="J30" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="K30" s="1" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="31" spans="1:14" ht="60" x14ac:dyDescent="0.25">
+      <c r="A31" s="1">
+        <v>30</v>
+      </c>
+      <c r="B31" s="1" t="s">
+        <v>105</v>
+      </c>
+      <c r="C31" s="1" t="s">
+        <v>107</v>
+      </c>
+      <c r="D31" s="1" t="s">
+        <v>113</v>
+      </c>
+      <c r="E31" s="1" t="s">
+        <v>106</v>
+      </c>
+      <c r="F31" s="1" t="s">
+        <v>55</v>
+      </c>
+      <c r="G31" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="H31" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="I31" s="1" t="s">
+        <v>114</v>
+      </c>
+      <c r="J31" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="K31" s="1" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="32" spans="1:14" ht="60" x14ac:dyDescent="0.25">
+      <c r="A32" s="1">
+        <v>31</v>
+      </c>
+      <c r="B32" s="1" t="s">
+        <v>105</v>
+      </c>
+      <c r="C32" s="1" t="s">
+        <v>107</v>
+      </c>
+      <c r="D32" s="1" t="s">
+        <v>115</v>
+      </c>
+      <c r="E32" s="1" t="s">
+        <v>106</v>
+      </c>
+      <c r="F32" s="1" t="s">
+        <v>55</v>
+      </c>
+      <c r="G32" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="H32" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="I32" s="1" t="s">
+        <v>116</v>
+      </c>
+      <c r="J32" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="K32" s="1" t="s">
+        <v>121</v>
       </c>
     </row>
   </sheetData>
+  <autoFilter ref="A1:K51" xr:uid="{00000000-0001-0000-0000-000000000000}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>